<commit_message>
chore(CWL): improve duplicate version error
</commit_message>
<xml_diff>
--- a/CustomWhateverLoader/package/LangMod/EN/~cwl_sources.xlsx
+++ b/CustomWhateverLoader/package/LangMod/EN/~cwl_sources.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\Elin.Plugins\CustomWhateverLoader\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7B439E7-6BE1-43F8-BC65-88CEF59F2B68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{927FDC62-00A5-4EDA-BF48-2052255E63FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17490" yWindow="975" windowWidth="28380" windowHeight="17610" tabRatio="555" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8295" yWindow="2985" windowWidth="25965" windowHeight="15615" tabRatio="555" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -983,17 +983,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Two versions of CWL are found!
-Only use the version that matches your game.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>cwl_warn_duplicate_cwl</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CWLのバージョンが2つ見つかりました！
-お使いのゲームに合ったバージョンのみを使用してください。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1800,6 +1790,18 @@
   </si>
   <si>
     <t>CWL/デバッグパネル</t>
+  </si>
+  <si>
+    <t>Two versions of CWL are found!
+Only use the version that matches your game.
+If you are using Nightly branch of Elin, remove Stable CWL.
+If you don't know what Nightly is, remove Nightly CWL.</t>
+  </si>
+  <si>
+    <t>CWLのバージョンが2つ見つかりました！
+お使いのゲームに合ったバージョンのみを使用してください。
+SteamでElinのNightlyブランチをお使いの場合は、Stable版のCWLを削除してください。
+Nightlyブランチがよくわからない場合は、Nightly版のCWLを削除してください。</t>
   </si>
 </sst>
 </file>
@@ -2374,10 +2376,10 @@
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="3" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="23.25">
@@ -2398,10 +2400,10 @@
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="23.25">
@@ -2413,7 +2415,7 @@
         <v>31</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="46.5">
@@ -2422,10 +2424,10 @@
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="3" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="46.5">
@@ -2434,10 +2436,10 @@
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="3" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="23.25">
@@ -2481,10 +2483,10 @@
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="23.25">
@@ -2493,10 +2495,10 @@
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="23.25">
@@ -2505,10 +2507,10 @@
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="23.25">
@@ -2517,10 +2519,10 @@
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="1" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="23.25">
@@ -2611,10 +2613,10 @@
       </c>
       <c r="B24" s="1"/>
       <c r="C24" s="1" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="23.25">
@@ -2623,10 +2625,10 @@
       </c>
       <c r="B25" s="1"/>
       <c r="C25" s="1" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="23.25">
@@ -2635,10 +2637,10 @@
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="1" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="23.25">
@@ -2815,10 +2817,10 @@
       </c>
       <c r="B41" s="1"/>
       <c r="C41" s="3" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="46.5">
@@ -3077,7 +3079,7 @@
         <v>208</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="23.25">
@@ -3089,7 +3091,7 @@
         <v>209</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="23.25">
@@ -3098,10 +3100,10 @@
       </c>
       <c r="B66" s="1"/>
       <c r="C66" s="9" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="46.5">
@@ -3110,10 +3112,10 @@
       </c>
       <c r="B67" s="1"/>
       <c r="C67" s="3" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="68" spans="1:4" s="10" customFormat="1" ht="23.25">
@@ -3146,10 +3148,10 @@
       </c>
       <c r="B70" s="1"/>
       <c r="C70" s="3" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="71" spans="1:4" s="10" customFormat="1" ht="23.25">
@@ -3290,10 +3292,10 @@
       </c>
       <c r="B82" s="1"/>
       <c r="C82" s="1" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="83" spans="1:4" ht="23.25">
@@ -3302,22 +3304,22 @@
       </c>
       <c r="B83" s="1"/>
       <c r="C83" s="3" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="84" spans="1:4" ht="51">
       <c r="A84" s="1" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B84" s="1"/>
       <c r="C84" s="3" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="85" spans="1:4" ht="25.5">
@@ -3326,22 +3328,22 @@
       </c>
       <c r="B85" s="1"/>
       <c r="C85" s="1" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="86" spans="1:4" ht="23.25">
       <c r="A86" s="1" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B86" s="1"/>
       <c r="C86" s="1" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="87" spans="1:4" ht="23.25">
@@ -3449,7 +3451,7 @@
         <v>159</v>
       </c>
       <c r="D95" s="14" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="96" spans="1:4" ht="23.25">
@@ -3461,7 +3463,7 @@
         <v>161</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="97" spans="1:4" ht="23.25">
@@ -3485,19 +3487,19 @@
         <v>165</v>
       </c>
       <c r="D98" s="14" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="99" spans="1:4" ht="23.25">
       <c r="A99" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B99" s="1"/>
       <c r="C99" s="25" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D99" s="9" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="100" spans="1:4" ht="23.25">
@@ -3578,10 +3580,10 @@
       </c>
       <c r="B106" s="1"/>
       <c r="C106" s="1" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="107" spans="1:4" ht="69.75">
@@ -3622,50 +3624,50 @@
     </row>
     <row r="110" spans="1:4" ht="23.25">
       <c r="A110" s="1" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B110" s="1"/>
       <c r="C110" s="20" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="111" spans="1:4" ht="46.5">
       <c r="A111" s="1" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B111" s="1"/>
       <c r="C111" s="3" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D111" s="3" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="112" spans="1:4" ht="25.5">
       <c r="A112" s="1" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B112" s="1"/>
       <c r="C112" s="22" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="113" spans="1:4" ht="23.25">
       <c r="A113" s="1" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B113" s="1"/>
       <c r="C113" s="21" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D113" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="114" spans="1:4" ht="23.25">
@@ -3686,10 +3688,10 @@
       </c>
       <c r="B115" s="15"/>
       <c r="C115" s="15" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="D115" s="15" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="116" spans="1:4" ht="23.25">
@@ -3698,10 +3700,10 @@
       </c>
       <c r="B116" s="15"/>
       <c r="C116" s="15" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="D116" s="15" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="117" spans="1:4" ht="25.5">
@@ -3746,322 +3748,322 @@
       </c>
       <c r="B120" s="15"/>
       <c r="C120" s="16" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="D120" s="16" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" ht="46.5">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" ht="139.5">
       <c r="A121" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B121" s="15"/>
       <c r="C121" s="16" t="s">
-        <v>218</v>
+        <v>347</v>
       </c>
       <c r="D121" s="16" t="s">
-        <v>216</v>
+        <v>346</v>
       </c>
     </row>
     <row r="122" spans="1:4" ht="25.5">
       <c r="A122" s="15" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B122" s="15"/>
       <c r="C122" s="19" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D122" s="15" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="123" spans="1:4" ht="23.25">
       <c r="A123" s="5" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B123" s="15"/>
       <c r="C123" s="15" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="D123" s="15" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="124" spans="1:4" ht="25.5">
       <c r="A124" s="15" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B124" s="15"/>
       <c r="C124" s="15" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="D124" s="15" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="125" spans="1:4" ht="69.75">
       <c r="A125" s="15" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B125" s="15"/>
       <c r="C125" s="23" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D125" s="16" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="126" spans="1:4" ht="51">
       <c r="A126" s="15" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B126" s="15"/>
       <c r="C126" s="24" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="D126" s="16" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="127" spans="1:4" ht="23.25">
       <c r="A127" s="15" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B127" s="15"/>
       <c r="C127" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D127" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="128" spans="1:4" ht="23.25">
       <c r="A128" s="15" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B128" s="15"/>
       <c r="C128" s="15" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D128" s="15" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="129" spans="1:4" ht="46.5">
       <c r="A129" s="12" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B129" s="15"/>
       <c r="C129" s="16" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="D129" s="16" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="130" spans="1:4" ht="23.25">
       <c r="A130" s="15" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B130" s="15"/>
       <c r="C130" s="15" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D130" s="15" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="131" spans="1:4" ht="23.25">
       <c r="A131" s="15" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B131" s="15"/>
       <c r="C131" s="15" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D131" s="15" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="132" spans="1:4" ht="46.5">
       <c r="A132" s="15" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B132" s="15"/>
       <c r="C132" s="16" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="D132" s="15" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="133" spans="1:4" ht="23.25">
       <c r="A133" s="15" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B133" s="15"/>
       <c r="C133" s="15" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="D133" s="15" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="134" spans="1:4" ht="23.25">
       <c r="A134" s="15" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B134" s="15"/>
       <c r="C134" s="15" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="D134" s="15" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="135" spans="1:4" ht="46.5">
       <c r="A135" s="15" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B135" s="15"/>
       <c r="C135" s="16" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="D135" s="16" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="136" spans="1:4" ht="23.25">
       <c r="A136" s="4" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B136" s="15"/>
       <c r="C136" s="15" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="D136" s="15" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="137" spans="1:4" ht="23.25">
       <c r="A137" s="15" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B137" s="15"/>
       <c r="C137" s="16" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="D137" s="16" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="138" spans="1:4" ht="46.5">
       <c r="A138" s="4" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B138" s="15"/>
       <c r="C138" s="16" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="D138" s="16" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="139" spans="1:4" ht="23.25">
       <c r="A139" s="4" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B139" s="15"/>
       <c r="C139" s="15" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="D139" s="15" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="140" spans="1:4" ht="46.5">
       <c r="A140" s="26" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B140" s="15"/>
       <c r="C140" s="16" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D140" s="16" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="141" spans="1:4" ht="46.5">
       <c r="A141" s="15" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="B141" s="15"/>
       <c r="C141" s="16" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="D141" s="16" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="142" spans="1:4" ht="93">
       <c r="A142" s="15" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B142" s="15"/>
       <c r="C142" s="16" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D142" s="16" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="143" spans="1:4" ht="23.25">
       <c r="A143" s="26" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B143" s="15" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C143" s="15"/>
       <c r="D143" s="15" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="144" spans="1:4" ht="23.25">
       <c r="A144" s="15" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B144" s="15" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C144" s="15"/>
       <c r="D144" s="15" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="145" spans="1:4" ht="23.25">
       <c r="A145" s="15" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B145" s="15" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C145" s="15"/>
       <c r="D145" s="15" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="146" spans="1:4" ht="23.25">
       <c r="A146" s="15" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="B146" s="15" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C146" s="15"/>
       <c r="D146" s="15" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="147" spans="1:4" ht="23.25">

</xml_diff>